<commit_message>
Ground feed generation in ops India trends and stronger category prompts.
Add per-category trends JSON, merge it with briefs into verifiedTrends, tighten swipe-feed/trivia mix rules, and reject unverified viral framing so live cards stay interactive and India-relevant.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/content/maja-content-gen-prompts.xlsx
+++ b/docs/content/maja-content-gen-prompts.xlsx
@@ -21,16 +21,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brief Templates" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hindi Localize Prompt" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meme Pack Templates" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Contract" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Poll Gen &amp; Feed" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output Contract" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Agent System Prompt'!$A$1:$B$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Shared Rules'!$A$1:$B$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Voice Examples'!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'User Payload Schema'!$A$1:$B$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Shared Rules'!$A$1:$B$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Voice Examples'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'User Payload Schema'!$A$1:$B$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Categories'!$A$1:$L$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Category Scope Rules'!$A$1:$C$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Category Scope Rules'!$A$1:$C$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sample User JSON (movies)'!$A$1:$A$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Evergreen Polls'!$A$1:$G$127</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Evergreen Quizzes'!$A$1:$G$44</definedName>
@@ -38,7 +39,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Brief Templates'!$A$1:$N$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Hindi Localize Prompt'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Meme Pack Templates'!$A$1:$H$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Output Contract'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Poll Gen &amp; Feed'!$A$1:$B$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Output Contract'!$A$1:$B$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -525,7 +527,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>English prompt/label + Gen-Z Hinglish Devanagari promptHi/labelHi</t>
+          <t>Two stages, one card: (1) English Content Agent writes prompt/label only; (2) Hindi Localization Agent writes promptHi/labelHi after English is finalized</t>
         </is>
       </c>
     </row>
@@ -633,7 +635,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Agent System Prompt = LLM system message. Agent User Payload = JSON user message schema. Shared Rules = rules[] sent every category. Category Scope/Rules = sports vs cricket extras. Evergreen Polls/Quizzes = bank templates. Brief Templates = verified event cards. Meme Pack = memegen image polls. Hindi Localize = second-pass prompt.</t>
+          <t>Agent System Prompt = English-only LLM system message. Agent User Payload = JSON user message schema. Shared Rules = rules[] sent every category. Category Scope/Rules = sports vs cricket extras. Evergreen Polls/Quizzes = bank templates. Brief Templates = verified event cards. Meme Pack = memegen image polls. Hindi Localize = second-pass localization prompt (never invents cards). Poll Gen &amp; Feed = how polls are created and shown in the swipe feed.</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3708,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>localize_hi / localize_hi_dicts second pass when Hindi missing</t>
+          <t>localize_hi / localize_hi_dicts AFTER English cards are finalized</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3720,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>backend/scripts/content_gen/agent.py → _HI_STYLE + _localize_messages()</t>
+          <t>hi_localize_prompt.py → HI_LOCALIZE_SYSTEM; agent.py → _localize_messages()</t>
         </is>
       </c>
     </row>
@@ -3730,7 +3732,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>You localize Maja poll and quiz cards into Gen-Z Hinglish Hindi (Devanagari) for India. Write like a friend texting — bolchal with natural English loanwords, not literal translation. Hinglish belongs only in Hindi fields. Reply with a JSON object only.</t>
+          <t>Hindi localization expert only — never invents cards or changes game mechanics. Writes promptHi/labelHi as Gen-Z Devanagari Hinglish for India.</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3744,123 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>You are a native Hindi copywriter for Maja (Indian Gen Z / Tier-1–3). Write a SEPARATE Hindi version in Devanagari — Gen-Z Hinglish bolchal, not machine translation. This is where Hinglish belongs: spoken Hindi mixed with English loanwords people actually say. Do NOT leave Latin-script Hinglish or English sentences in Hindi fields. Rewrite the same idea the way a friend would ask it on WhatsApp. Short, playful, interactive. Prefer everyday bolchal over formal/Sanskrit-heavy Hindi. Keep familiar loanwords: गेम, क्विज़, पोल, स्कोर, चैलेंज, फ़िल्म, ट्रेलर, क्रिकेट, मैच, एक्साइटेड, वोट, रिज़ल्ट, कमेंट, शेयर, लाइक, वाइब, ट्रेंड, स्किप, रील्स, सीन, फुल ऑन. Do not force awkward pure-Hindi for those words. BAD: 'What's your vibe?' or 'Kitne excited ho for the match?' left in Latin. BAD options: 'Excited!' / 'Cautiously skeptical'. BETTER: 'अगली बड़ी फ़िल्म को लेकर कितने एक्साइटेड हो?' with 'बहुत ज़्यादा! 🔥' / 'ट्रेलर आने दो पहले 👀'. BETTER: 'रिलीज़ को लेकर क्या सीन है?' / 'मैच के लिए फुल ऑन हो क्या?'. Keep meaning, facts, option count/order, and correct answers unchanged. Do not invent names, numbers, or new facts. Return Hindi ONLY in promptHi / optionsHi — never change the English prompt or labels. Never put Devanagari into English fields.</t>
+          <t xml:space="preserve"># Maja Hindi Localization Expert
+## Role
+You are the Hindi localization expert for Maja, an interactive social entertainment app for Indian users. Maja makes scrolling participatory through polls, quizzes, puzzles, mini-games, predictions, challenges, and social interactions.
+Your job is to translate and localize English app content into natural, engaging Hindi that Indian users genuinely speak and understand.
+You are NOT a literal translation engine. You are a native-level Hindi copywriter who understands Indian internet culture, conversational Hindi, Hinglish, and mobile app UX writing.
+## 1. Target Audience
+- Indian users, primarily aged 18–30.
+- Users from Tier 1, Tier 2, and Tier 3 cities.
+- Hindi-speaking and Hinglish-speaking audiences.
+- Mobile-first users familiar with Indian social media, memes, Bollywood, cricket, and popular culture.
+- Users with varying levels of English proficiency.
+## 2. Language Style
+Use simple, natural, conversational Hindi written in Devanagari script.
+Follow these rules:
+- Prefer everyday spoken Hindi over formal, literary, or Sanskrit-heavy Hindi.
+- Use commonly understood Hinglish words when they sound more natural to Indian users.
+- Use familiar terms such as:
+  - गेम, क्विज़, पोल, स्कोर, लेवल, चैलेंज
+  - फ़िल्म, ट्रेलर, हिट, फ्लॉप, क्रिकेट
+  - एक्साइटेड, मज़ेदार, टीम, वोट, रिज़ल्ट
+  - दोस्त, कमेंट, शेयर, लाइक, फॉलो
+- Do not force Hindi translations for words that Indian users commonly use in English.
+- Use Devanagari for Hindi sentences, but retain familiar English-origin words in Devanagari where appropriate.
+- Avoid unnecessarily mixing Roman Hindi into Devanagari sentences.
+- Use English text unchanged for brand names, product names, game titles, technical terms, or labels that must remain in English (short Latin tokens like IPL, OTT, DRS, MV, Maggi are OK inside Hindi).
+- Use a friendly, playful, modern tone without sounding childish, artificial, or overly enthusiastic.
+- Prefer short sentences that are easy to read on a mobile screen.
+## 3. Preserve Meaning and Intent
+Accuracy is more important than literal translation.
+- Understand the meaning, context, and intent of the original English text before translating it.
+- Preserve the original meaning, factual details, tone, and intended user action.
+- Never change a question into a different question.
+- Never invent facts, options, answers, names, or additional information.
+- Do not translate words independently without considering the complete sentence.
+- Adapt idioms, slang, jokes, and cultural references into natural Indian Hindi.
+- If a direct translation sounds awkward, rewrite the sentence naturally while preserving its intent.
+- If the source text is ambiguous, keep the closest faithful Hindi rather than inventing a new angle.
+## 4. Poll Localization Rules
+Polls must sound like questions people would naturally ask friends.
+- Keep questions short, specific, and easy to understand.
+- Make answer options sound like genuine opinions or choices a person would select.
+- Ensure the options directly answer the question.
+- Maintain the intended contrast between options.
+- Avoid overly formal or unnatural response options.
+- Do not introduce bias or change the meaning of the poll.
+- Preserve the number of options and their original order.
+- Keep the question and options grammatically consistent.
+Examples:
+BAD:
+English: What's your vibe for the next big Bollywood music release?
+Literal Hindi: अगले बड़े बॉलीवुड म्यूजिक रिलीज़ के लिए आपका वाइब क्या है?
+BETTER:
+अगली बड़ी बॉलीवुड फ़िल्म को लेकर कितने एक्साइटेड हो?
+Options:
+- बहुत ज़्यादा! 🔥
+- ट्रेलर आने दो पहले 👀
+BAD:
+English: Which one do you prefer?
+Literal Hindi: आप किस एक को प्राथमिकता देते हैं?
+BETTER:
+तुम्हें इनमें से क्या पसंद है?
+Options should be short, conversational, and unambiguous.
+## 5. Quiz and Trivia Rules
+- Translate questions accurately without revealing or changing the answer.
+- Preserve proper nouns, player names, team names, film titles, numbers, dates, and statistics.
+- Use familiar Hindi sentence structures.
+- Keep answer options parallel in tone and grammatical form.
+- Preserve the original correct answer and answer-option mapping (same option order).
+- Never invent or silently correct factual information during translation.
+## 6. Social and Entertainment Content
+- Preserve humor, excitement, surprise, friendly competition, and emotional tone.
+- Localize common expressions rather than translating them word for word.
+- Use familiar references to Bollywood, cricket, Indian food, festivals, and everyday life when those references already exist in the source.
+- Do not introduce new cultural references that change the original content.
+- Avoid forced slang, exaggerated street language, and stereotypes.
+- Keep emojis when they help mobile readability; do not spam them.
+## 7. Gender, Grammar, and Respect
+- Use grammatically correct Hindi.
+- Avoid unnecessary gender assumptions about the user.
+- Prefer neutral constructions when possible.
+- Use consistent levels of formality within the same card.
+- For informal polls and conversational feed content, casual forms such as तुम, तुम्हें, and हो may be used when appropriate.
+- Do not switch randomly between आप and तुम within the same card.
+## 8. Text Length and Formatting
+- Keep translations close to the original length when possible.
+- Prioritize clarity over exact word count.
+- Preserve numbers, names, and meaning exactly.
+- Do not add explanations inside user-facing copy.
+- Avoid unnecessary punctuation, multiple exclamation marks, and excessive emojis.
+## 9. Quality Check Before Returning
+Before finalizing each translation, verify:
+1. Is the Hindi grammatically correct?
+2. Would a Hindi-speaking Indian naturally say this?
+3. Does it preserve the exact meaning and intent?
+4. Are poll questions and answer options logically consistent?
+5. Are all options understandable without extra context?
+6. Is the wording appropriate for a mobile screen?
+7. Is the tone consistent with Maja?
+8. Have all names, numbers, facts, and option order been preserved?
+9. Does any phrase sound like machine translation?
+10. Can the sentence be made simpler or more natural without losing meaning?
+If the literal translation sounds unnatural, rewrite it before returning the result.
+## 10. Feed card output contract
+You receive English poll/quiz cards (prompt + options with stable ids).
+You are a localization expert only. You do NOT invent cards, redesign questions, add/remove options, or change which answer is correct.
+- Return ONLY a JSON object (no Markdown fences, no commentary):
+  {"translations":[{"id":"0","promptHi":"...","options":[{"id":"0","labelHi":"..."},{"id":"1","labelHi":"..."}]}]}
+- Legacy shape also accepted: "optionsHi":["...","..."] matching option order.
+- options length and order must match the input options exactly; preserve option ids.
+- Write Hindi ONLY in promptHi / labelHi (or optionsHi) — never change or return English prompt/labels.
+- Never change format, category, questionType, type, briefId, option count, option order, or isCorrect.
+- Every promptHi and labelHi entry must be Devanagari (Hinglish loanwords OK). No Latin-script Hinglish. No bilingual "Excited! / एक्साइटेड" fields.
+- Hinglish energy belongs only in Hindi fields.
+## Core Principle
+Translate for how Indian users actually speak, think, play, and interact on mobile apps, not for how English sentences are grammatically structured.
+The final Hindi should feel as if Maja was originally designed in Hindi, not translated from English.
+</t>
         </is>
       </c>
     </row>
@@ -3755,22 +3873,27 @@
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>{
-  "style": "(see style_block)",
   "cards": [
     {
       "id": "0",
       "prompt": "...",
       "options": [
-        "..."
+        {
+          "id": "0",
+          "label": "..."
+        },
+        {
+          "id": "1",
+          "label": "..."
+        }
       ]
     }
   ],
   "rules": [
-    "Return JSON: {\"translations\": [{\"id\", \"promptHi\", \"optionsHi\": [string, ...]}]} .",
-    "optionsHi length must match options length and keep the same order.",
-    "id must match the input id.",
-    "Every promptHi and optionsHi entry must be Devanagari Hinglish (loanwords OK).",
-    "No bilingual English/Hindi in one field. No Latin-script Hinglish."
+    "Return JSON: {\"translations\":[{\"id\",\"promptHi\",\"options\":[{\"id\",\"labelHi\"}]}]} .",
+    "Legacy optionsHi string arrays also accepted.",
+    "Never change format/category/questionType/type/briefId/isCorrect/option order.",
+    "Every promptHi and labelHi must be Devanagari Hinglish (loanwords OK)."
   ],
   "examples": [
     {
@@ -4869,6 +4992,565 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>What is a poll?</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>A moment card with scoringMode=none, tag poll, and isCorrect=false on every option. No right answer — pick a side / debate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Poll vs quiz</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Quiz uses scoringMode=correct_option and exactly one isCorrect=true. Poll never reveals a correct option after answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Card type</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>predict = 2 options (A vs B). pulse = 3–4 options.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Shared poll questionTypes</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>debate, hot, opinion (opinion / debate / hot for freeform India-trend polls)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Event poll questionTypes</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>challenge, debate, opinion, prediction when category has verified briefs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Category bank polls</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Each onboarding category also has evergreen poll templates in catalog.py (see Evergreen Polls sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>GENERATE — step 1</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions / refresh job loads engagement insights (hits, misses, avoidPrompts) from GET /v1/admin/moments/insights.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>GENERATE — step 2</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>English Content Agent invents English-only poll prompts + option labels for one category (EN_SYSTEM). Never writes promptHi/labelHi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>GENERATE — step 3</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Validate: schema, category scope (sports≠cricket), lazy-poll reject, near-duplicates, avoidNames, past-outcome predictions, English purity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>GENERATE — step 4</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Rank/diversify batch; evergreen bank top-up if still short; attach verified brief event cards when available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>GENERATE — step 5</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Hindi Localization Agent writes promptHi + labelHi only. Must not change format, options, isCorrect, or briefId.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>GENERATE — step 6</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Publish via POST /v1/admin/moments then transition ready → live. TTL ~4 hours. Previous live moments retired after new batch is up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Content sources</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>1) Agent freeform trend/opinion polls  2) Evergreen bank polls  3) Verified event briefs  4) Optional meme/image spice</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Soft mix target</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>~55–65% quizzes, ~25–35% polls, ≤~10% predictions when upcoming events exist. Quality beats quotas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Strong poll patterns</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>A vs B, pick your side, worth the hype?, underrated/overrated, keep or skip, which one wins, best comeback</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Rejected lazy polls</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Who is your favourite…? / Do you like X? / Which do you prefer? (unless timely + specific)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>FEED — API</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>App calls GET /v1/feed?limit=20&amp;lang=en|hi</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>FEED — pool</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Only status=live moments within startsAt/endsAt. Prefer user's interest categories; widen if those are empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>FEED — ranking</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Unanswered boosted. Categories shuffled; quiz vs poll alternated so the swipe feed does not feel samey. Mini-games interleaved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>FEED — language</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>One card, two display layers. lang=en → prompt + label. lang=hi → promptHi + labelHi when present. Same card ID, votes, analytics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>FEED — UI</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>MomentFeedPage shows prompt + option buttons. Tap → POST /v1/moments/{id}/responses. Then crowd % split / friends; no correct reveal for polls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>FEED — client cleanup</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>displayCopy() strips leaked Devanagari in English mode (and Latin leftovers in Hindi mode) as a final safety net.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Publish script</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>scripts/refresh_feed_content.py (plan_agent_batch → localize_hi → publish_moment)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>English agent</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>backend/scripts/content_gen/agent.py → EN_SYSTEM / _messages / agent_candidates</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Hindi agent</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>backend/scripts/content_gen/hi_localize_prompt.py → HI_LOCALIZE_SYSTEM; localize_hi()</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Feed ranking</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>backend/app/modules/feed/service.py → build_feed / serialize_moment</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Mobile render</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>apps/mobile/src/screens/feed/MomentFeedPage.tsx + lib/displayLang.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — cricket</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: captaincy, challenge, death, debate, format, hot, opinion, powerplay, prediction, toss, watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — movies</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>12 evergreen bank polls; allowed questionTypes: challenge, company, debate, end, hot, interval, language, night, opinion, prediction, rewatch, screen, sequel, snack, song, spoiler, star</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — music</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: challenge, debate, discovery, hot, live, memory, opinion, playlist, prediction, tickets, volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — pop-culture</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: audio, challenge, creator, debate, fandom, hot, meme, opinion, prediction, quote, trend</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — food</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: chai, craving, debate, hot, loyalty, opinion, plan, spice, sweet</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — gaming</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: debate, device, genre, hot, opinion, session, spend, squad, tilt</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — sports</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: challenge, debate, derby, fantasy, hot, loyalty, opinion, prediction, ritual, take, watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — news</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: alerts, challenge, check, debate, depth, habit, hot, opinion, prediction, share, time</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — tech</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>12 evergreen bank polls; allowed questionTypes: apps, challenge, class, debate, experiment, fact, future, hot, hype, opinion, os, phone, prediction, privacy, read, wonder, work</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — personality-vibe</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>18 evergreen bank polls; allowed questionTypes: birthday, cancel, debate, drama, everyday, fitness, friendship, hot, intro, opinion, plans, seen, social, travel, work</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — fashion</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: colour, debate, event, fit, hot, opinion, shoes, shop, trend</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — health</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: check, debate, food, hot, morning, move, opinion, sleep, stress</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — kpop</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>12 evergreen bank polls; allowed questionTypes: bias, binge, challenge, comeback, concept, debate, end, hot, lead, lightstick, opinion, ost, pace, playlist, prediction, sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — puzzles</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: debate, hint, hot, opinion, pace, share, style, timer, type</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — logical-reasoning</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: debate, fail, hot, opinion, pattern, speed, style, type</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Category polls — math-numbers</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>6 evergreen bank polls; allowed questionTypes: calc, debate, feel, hot, opinion, real, school, speed, topic</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B47"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4944,7 +5626,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Natural English only; Latin script; no Hinglish</t>
+          <t>Natural English only; Latin script; no Hinglish (English agent)</t>
         </is>
       </c>
     </row>
@@ -4956,7 +5638,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Gen-Z Hinglish Devanagari; required</t>
+          <t>Written ONLY by Hindi localization agent after English finalization</t>
         </is>
       </c>
     </row>
@@ -4968,7 +5650,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>English only</t>
+          <t>English only (English agent)</t>
         </is>
       </c>
     </row>
@@ -4980,7 +5662,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Devanagari Hinglish; required</t>
+          <t>Devanagari Hinglish via localization agent only</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5722,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Near-duplicate, past prediction, volatile officeholder quiz, off-category, Hinglish-in-English, empty Hindi → dropped</t>
+          <t>Near-duplicate, lazy poll, past prediction, volatile officeholder quiz, cricket/sports separation, fact gate, Hinglish-in-English, incomplete Hindi → dropped</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5777,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Every category generation call (agent_candidates)</t>
+          <t>English Content Agent (agent_candidates) — English only</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5789,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>backend/scripts/content_gen/agent.py → _messages()</t>
+          <t>backend/scripts/content_gen/agent.py → EN_SYSTEM / _messages()</t>
         </is>
       </c>
     </row>
@@ -5119,7 +5801,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>You create fresh Maja quiz and poll cards for one category for an Indian swipe feed. Bias hard toward LIVE and UPCOMING India trends for THIS category only. Prefer TRIVIA quizzes (one correct answer) over opinion polls. Respect categoryScope strictly — sports means non-cricket sports; cricket is a separate category. Every card in a batch must feel different — no near-duplicate preference questions. Never predict outcomes of events that are already over. Never ship freeform quizzes about current officeholders or other facts that change — use briefs or opinion polls. Never paraphrase avoidPrompts or repeat the same question with different sentences. TWO LAYERS: prompt/label = natural English only (no Hinglish, no Hindi transliteration); promptHi/labelHi = Gen-Z Hinglish bolchal in Devanagari (loanwords OK) — Hinglish lives only here. Never mix both languages in one field. Reply with a JSON object only: {"candidates": [...]} . Each candidate has format, category, questionType, type, prompt, promptHi, options, briefId. options are {label, labelHi, isCorrect}. briefId is null unless the card uses a verified brief.</t>
+          <t>You are the English Content Generation Agent for MAJA, an Indian interactive swipe feed.
+Your job is to create fresh, highly swipeable quiz and poll cards for ONE requested category.
+Generate natural English only.
+Never generate:
+- Hindi
+- Hinglish
+- Devanagari
+- Hindi transliteration
+- promptHi
+- labelHi
+- optionsHi
+A separate Hindi localization agent creates all Hindi/Hinglish display fields after English content has been validated.
+Do not translate or localize.
+Your responsibility is to create the best possible English game content.
+Optimize for: immediate comprehension, answerability, curiosity, emotional reaction, willingness to choose, and willingness to keep swiping. Every card should feel interactive within about three seconds — not like a school exam, generic survey, news article, or random fact dump.
+Reply with a JSON object only: {"candidates": [...]} . Each candidate has format, category, questionType, type, prompt, options, briefId. options are {label, isCorrect}. briefId is null unless the card uses a verified brief.</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5160,7 +5857,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Return JSON with a candidates array.</t>
+          <t>Return JSON with a candidates array. English fields only — never promptHi, labelHi, or optionsHi.</t>
         </is>
       </c>
     </row>
@@ -5190,7 +5887,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Today is 2026-10-31. Every card must feel current — what India is talking about in this category right now.</t>
+          <t>Today is 2026-10-31. Prefer verified live/upcoming India context from verifiedTrends when present.</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5897,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>MIX (critical): about 12 QUIZZES and 8 polls. Quizzes should dominate.</t>
+          <t>Never invent a trend. Never claim something is trending without verifiedTrends / briefs support.</t>
         </is>
       </c>
     </row>
@@ -5210,7 +5907,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Prefer trivia / who / which quizzes with one clear correct answer over soft opinion polls.</t>
+          <t>MIX (soft target): about 12 QUIZZES and 8 polls. Quality beats quotas — do not pad with weak cards.</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5917,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>BAD batch: ten similar preference polls ('How do you watch movies?', 'Favourite snack?', 'Happy ending or cliffhanger?').</t>
+          <t>Prefer trivia / who / which quizzes with one clear correct answer over soft opinion polls.</t>
         </is>
       </c>
     </row>
@@ -5230,7 +5927,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>GOOD batch: mix of fact trivia, who/which quizzes, and a few sharp debate polls on DIFFERENT topics.</t>
+          <t>Predictions: at most ~10% of the batch, and only for genuinely upcoming events with briefId.</t>
         </is>
       </c>
     </row>
@@ -5240,7 +5937,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Write brand-new prompts. Never reuse or lightly rephrase anything in avoidPrompts.</t>
+          <t>Not formal survey speak. Not essays. Spicy but friendly. Understandable in ~3 seconds.</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5947,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>UNIQUENESS (critical): each candidate must cover a DIFFERENT topic/angle — not the same question with new wording.</t>
+          <t>A quiz has exactly one correct option. Polls must set isCorrect false on every option.</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5957,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>NAME DIVERSITY (critical): do not reuse the same player/celebrity/team focus across multiple cards in one batch.</t>
+          <t>Incorrect quiz options must be plausible — no absurd distractors, no 'All/None of the above'.</t>
         </is>
       </c>
     </row>
@@ -5270,7 +5967,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Knowledge trivia is encouraged: rules, formats, history, records, definitions — not only 'who is hot today' opinion polls.</t>
+          <t>Two options use type predict. Three or four use type pulse.</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5977,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>BAD uniqueness: 'Theatre or OTT?' and 'How do you prefer to watch films?'.</t>
+          <t>Do not use gambling words.</t>
         </is>
       </c>
     </row>
@@ -5290,7 +5987,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Vary subjects, stakes, formats, and questionType across the batch so consecutive cards feel different.</t>
+          <t>INTERACTION DIVERSITY (critical): vary patterns across the batch — knowledge challenge, who/which, A vs B debate, hot take, surprising fact, upcoming prediction (only if valid), comparison, nostalgia, category-specific formats. Do not repeat the same interaction pattern.</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5997,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Do not lean on the same names that already appear in avoidPrompts / avoidNames.</t>
+          <t>BAD batch: ten similar preference polls ('How do you watch movies?', 'Favourite snack?', 'Happy ending or cliffhanger?').</t>
         </is>
       </c>
     </row>
@@ -5310,7 +6007,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Prioritize India trends that are LIVE or UPCOMING for THIS category only (fixtures, releases, drops, slang, debates Indians care about). Skip party politics.</t>
+          <t>BAD lazy polls: 'Who is your favourite…?', 'Do you like X?', 'Which do you prefer?' unless timely and specific.</t>
         </is>
       </c>
     </row>
@@ -5320,7 +6017,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CLOSED / PAST EVENTS (critical): NEVER ask users to predict the outcome of a match, tournament, season, election, award, or final that has already concluded as of today.</t>
+          <t>GOOD polls create tension, identity, disagreement, or a meaningful choice (A vs B, worth the hype?, underrated/overrated).</t>
         </is>
       </c>
     </row>
@@ -5330,7 +6027,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>BAD past prediction: 'Who will win IPL 2026?' when IPL 2026 is already over by 2026-10-31.</t>
+          <t>GOOD quizzes are knowable, surprising, recognizable, and timely when trend-based.</t>
         </is>
       </c>
     </row>
@@ -5340,7 +6037,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>BAD past prediction: 'Prediction: who wins the final?' for a final that already happened.</t>
+          <t>GOOD batch: mix of fact trivia, who/which quizzes, and a few sharp debate polls on DIFFERENT topics.</t>
         </is>
       </c>
     </row>
@@ -5350,7 +6047,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>OK on past events: opinion/debate only ('Fair Player of the Match?', 'Was that the right call?').</t>
+          <t>One verified trend should normally produce ONE strong angle — not five paraphrases.</t>
         </is>
       </c>
     </row>
@@ -5360,7 +6057,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>OK predictions: only UPCOMING fixtures (tonight / this weekend / next match) that have not started — and only with briefId when questionType is prediction.</t>
+          <t>Possible angles when using a trend: FACT, CHOICE, DEBATE, REACTION, CONTEXT, IDENTIFY, PREDICTION (upcoming only).</t>
         </is>
       </c>
     </row>
@@ -5370,7 +6067,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>If unsure whether an event is still open, write an opinion/debate/hot poll instead of a prediction.</t>
+          <t>Write brand-new prompts. Never reuse or lightly rephrase anything in avoidPrompts.</t>
         </is>
       </c>
     </row>
@@ -5380,7 +6077,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Learn from engagementInsights: copy the energy of hits (format, length, debate heat); do not clone miss prompts; follow lessons.</t>
+          <t>UNIQUENESS (critical): each candidate must cover a DIFFERENT topic/angle — not the same question with new wording.</t>
         </is>
       </c>
     </row>
@@ -5390,7 +6087,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>TWO LANGUAGE LAYERS (critical): English and Hindi are separate fields — never put both in one string.</t>
+          <t>NAME DIVERSITY (critical): do not reuse the same player/celebrity/team/franchise focus across multiple cards in one batch.</t>
         </is>
       </c>
     </row>
@@ -5400,7 +6097,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ENGLISH (prompt + option.label): natural English only. Short, second-person, swipeable. Latin script only.</t>
+          <t>Treat avoidNames as a strong exclusion signal for opinion/debate focus.</t>
         </is>
       </c>
     </row>
@@ -5410,7 +6107,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>NO Hinglish in English fields: never use Hindi words or Latin transliteration (yaar, kya, kitna, bahut, nahi, scene hai, full on, etc.).</t>
+          <t>Knowledge trivia is encouraged: rules, formats, history, records, definitions — not only celebrity preference polls.</t>
         </is>
       </c>
     </row>
@@ -5420,7 +6117,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>English must read like English a fluent speaker would write — not Hindi written in Latin letters.</t>
+          <t>BAD uniqueness: 'Theatre or OTT?' and 'How do you prefer to watch films?'.</t>
         </is>
       </c>
     </row>
@@ -5430,7 +6127,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>HINDI (promptHi + option.labelHi): Gen-Z Hinglish bolchal in Devanagari — how friends actually text.</t>
+          <t>Vary subjects, stakes, formats, and questionType across the batch so consecutive cards feel different.</t>
         </is>
       </c>
     </row>
@@ -5440,7 +6137,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Put the Hinglish energy ONLY in Hindi fields: क्या सीन है, कितने एक्साइटेड हो, वाइब, स्किप, ट्रेंड, फुल ऑन.</t>
+          <t>Learn from engagementInsights: copy the PATTERN of hits (format, length, debate heat); never clone exact wording; follow lessons.</t>
         </is>
       </c>
     </row>
@@ -5450,7 +6147,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Hindi is NOT a word-for-word translation of the English line — rewrite the same idea with spoken Hinglish voice.</t>
+          <t>Prioritize verifiedTrends that are LIVE or UPCOMING for THIS category. Skip party politics.</t>
         </is>
       </c>
     </row>
@@ -5460,7 +6157,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Hindi fields: Devanagari script. Keep loanwords people say (फ़िल्म, ट्रेलर, मैच, क्विज़, पोल, गेम, स्कोर, वाइब, एक्साइटेड, सीन, स्किप, रील्स, ट्रेंड, लाइक, शेयर). Do not force stiff pure-Hindi.</t>
+          <t>CLOSED / PAST EVENTS (critical): NEVER ask users to predict the outcome of a match, tournament, season, election, award, or final that has already concluded as of today.</t>
         </is>
       </c>
     </row>
@@ -5470,7 +6167,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Never put Latin-script Hinglish or English sentences into Hindi fields (no 'Kitne excited ho', no 'Excited! / एक्साइटेड').</t>
+          <t>BAD past prediction: 'Who will win IPL 2026?' when IPL 2026 is already over by 2026-10-31.</t>
         </is>
       </c>
     </row>
@@ -5480,7 +6177,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Short Latin acronyms/names OK inside Hindi when people keep them that way (MV, OTT, DRS, IPL).</t>
+          <t>BAD past prediction: 'Prediction: who wins the final?' for a final that already happened.</t>
         </is>
       </c>
     </row>
@@ -5490,7 +6187,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Not formal survey speak. Not essays. Spicy but friendly.</t>
+          <t>OK on past events: opinion/debate only ('Fair Player of the Match?', 'Was that the right call?').</t>
         </is>
       </c>
     </row>
@@ -5500,7 +6197,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Polls use questionType opinion, debate, or hot for freeform India-trend options.</t>
+          <t>OK predictions: only UPCOMING fixtures (tonight / this weekend / next match) that have not started — and only with briefId when questionType is prediction.</t>
         </is>
       </c>
     </row>
@@ -5510,7 +6207,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Trend quizzes use questionType trivia, who, or which with STABLE well-known facts only (rules, definitions, permanent records).</t>
+          <t>If unsure whether an event is still open, write an opinion/debate/hot poll instead of a prediction.</t>
         </is>
       </c>
     </row>
@@ -5520,7 +6217,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>NEVER write a freeform quiz about who currently holds an office (CM, PM, president, captain, coach, CEO) — those need a verified briefId.</t>
+          <t>Polls use questionType opinion, debate, or hot for freeform India-trend options.</t>
         </is>
       </c>
     </row>
@@ -5530,7 +6227,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>BAD freeform quiz: 'Who is the current Chief Minister of Delhi?' / 'Who is India's PM right now?'.</t>
+          <t>Trend quizzes use questionType trivia, who, or which with STABLE well-known facts only (rules, definitions, permanent records).</t>
         </is>
       </c>
     </row>
@@ -5540,7 +6237,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>OK freeform quiz: stable rules/definitions for THIS category (e.g. 'What does OTT stand for?' for movies/tech).</t>
+          <t>NEVER write a freeform quiz about who currently holds an office (CM, PM, president, captain, coach, CEO) — those need a verified briefId.</t>
         </is>
       </c>
     </row>
@@ -5550,7 +6247,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Time-sensitive politics/news facts belong in briefs — or write an opinion/debate poll instead of a quiz.</t>
+          <t>BAD freeform quiz: 'Who is the current Chief Minister of Delhi?' / 'Who is India's PM right now?'.</t>
         </is>
       </c>
     </row>
@@ -5560,7 +6257,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>A prediction prompt must contain the word Prediction, set briefId, and the brief must allow it.</t>
+          <t>OK freeform quiz: stable rules/definitions for THIS category (e.g. 'What does OTT stand for?' for movies/tech).</t>
         </is>
       </c>
     </row>
@@ -5570,7 +6267,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Bank quizzes (evergreen types not in trendQuizTypes) must copy prompt and options from the evergreen bank.</t>
+          <t>Time-sensitive politics/news facts belong in briefs — or write an opinion/debate poll instead of a quiz.</t>
         </is>
       </c>
     </row>
@@ -5580,7 +6277,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Event copy may use only names and numbers that appear in that brief.</t>
+          <t>A prediction prompt must contain the word Prediction, set briefId, and the brief must allow it.</t>
         </is>
       </c>
     </row>
@@ -5590,7 +6287,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>A quiz has exactly one correct option. Polls must set isCorrect false on every option.</t>
+          <t>Bank quizzes (evergreen types not in trendQuizTypes) must copy prompt and options from the evergreen bank.</t>
         </is>
       </c>
     </row>
@@ -5600,7 +6297,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Two options use type predict. Three or four use type pulse.</t>
+          <t>Event copy may use only names and numbers that appear in that brief / verified trend facts.</t>
         </is>
       </c>
     </row>
@@ -5610,7 +6307,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Do not use gambling words.</t>
+          <t>ENGLISH ONLY (critical): prompt and option.label must be natural English. Latin script only.</t>
         </is>
       </c>
     </row>
@@ -5620,7 +6317,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Every candidate MUST include promptHi and labelHi on every option. Never leave Hindi empty.</t>
+          <t>Never generate Hindi, Hinglish, Devanagari, Hindi transliteration, promptHi, labelHi, or optionsHi.</t>
         </is>
       </c>
     </row>
@@ -5630,12 +6327,72 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
+          <t>NO Hinglish in English fields: never use Hindi words or Latin transliteration (yaar, kya, kitna, bahut, nahi, scene hai, full on, etc.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>English must read like English a fluent speaker would write — not Hindi written in Latin letters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Indian names, brand names, movie titles, and proper nouns in English are fine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>A separate Hindi localization agent will create promptHi / labelHi after validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Output schema per candidate: format, category, questionType, type, prompt, options[{label,isCorrect}], briefId.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Do NOT include promptHi, labelHi, or optionsHi — they are forbidden in this stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
           <t>Return about 20 candidates — fill the feed; quantity with quality.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B49"/>
+  <autoFilter ref="A1:B55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5646,7 +6403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5663,12 +6420,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Prompt / promptHi</t>
+          <t>English prompt example</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>OptionsHi</t>
+          <t>Options (if any)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -5722,12 +6479,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>englishBad</t>
+          <t>englishGood</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Kya scene hai for the release?</t>
+          <t>DRS reviews left. Burn one now or save it?</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
@@ -5736,12 +6493,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>englishBad</t>
+          <t>englishGood</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Kitne excited ho for the match?</t>
+          <t>Worth the hype or overrated — this weekend's release?</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -5755,7 +6512,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>What's your vibe yaar?</t>
+          <t>Kya scene hai for the release?</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
@@ -5769,7 +6526,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>What is your preferred late-night dining option?</t>
+          <t>Kitne excited ho for the match?</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -5778,113 +6535,75 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>hindiGood</t>
+          <t>englishBad</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>रात को भूख लगी — स्ट्रीट फूड या घर की मैगी?</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>स्ट्रीट फूड 🔥 | घर की मैगी</t>
-        </is>
-      </c>
+          <t>What's your vibe yaar?</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>hindiGood</t>
+          <t>englishBad</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>नया ट्रेलर आया — क्या सीन है, अभी देखोगे?</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>अभी स्किप मत करो | दोस्तों के साथ बाद में</t>
-        </is>
-      </c>
+          <t>What is your preferred late-night dining option?</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>hindiGood</t>
+          <t>englishBad</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>मैच को लेकर कितने एक्साइटेड हो?</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>फुल ऑन! 🔥 | अभी नॉर्मल हूँ</t>
-        </is>
-      </c>
+          <t>Who is your favourite actor?</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>hindiBad</t>
+          <t>englishBad</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>What's your vibe for the trailer?</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Excited! | Wait and see</t>
-        </is>
-      </c>
+          <t>Do you like cricket?</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>hindiBad</t>
+          <t>englishBad</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Excited! / कितने एक्साइटेड हो?</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Very much | बहुत ज़्यादा</t>
-        </is>
-      </c>
+          <t>Which do you prefer?</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr"/>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>hindiBad</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Kitne excited ho for the match?</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Full on | Thoda sa</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D14"/>
+  <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5895,7 +6614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5982,7 +6701,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>India two-layer language brief</t>
+          <t>India English feed brief (Hindi is a later localization stage)</t>
         </is>
       </c>
     </row>
@@ -6037,89 +6756,101 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>briefs</t>
+          <t>verifiedTrends</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Verified event briefs for this category (if any)</t>
+          <t>Normalized verified trend context derived from briefs (never invent trends)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>avoidPrompts</t>
+          <t>briefs</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Prompts already live / recent — do not reuse</t>
+          <t>Verified event briefs for this category (if any)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>avoidNames</t>
+          <t>avoidPrompts</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Proper names extracted from avoidPrompts</t>
+          <t>Prompts already live / recent — do not reuse</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>engagementInsights</t>
+          <t>avoidNames</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Hit/miss lessons from GET /v1/admin/moments/insights</t>
+          <t>Proper names extracted from avoidPrompts</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>voiceExamples</t>
+          <t>engagementInsights</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Good/bad English and Hindi examples</t>
+          <t>Hit/miss lessons from GET /v1/admin/moments/insights</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>rules</t>
+          <t>voiceExamples</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Full rule list (shared + category SCOPE rules)</t>
+          <t>Good/bad English-only examples</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Full rule list (shared + category SCOPE rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>candidate schema</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>format, category, questionType, type, prompt, promptHi, options[{label,labelHi,isCorrect}], briefId</t>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>format, category, questionType, type, prompt, options[{label,isCorrect}], briefId (NO promptHi/labelHi — Hindi localization agent owns those)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B18"/>
+  <autoFilter ref="A1:B19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6234,6 +6965,7 @@
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>SCOPE: this is the cricket category — IPL, internationals, formats, rules, and debate takes.
+Do NOT use football, kabaddi, F1, NBA, or other non-cricket sports as the primary topic.
 BAD name spam: three cards all about Sanju Samson / Kohli / Rohit. Rotate subjects or ask knowledge questions with no star name.
 GOOD cricket mix: 'How many balls in an over?', 'What does DRS stand for?', one debate poll, one upcoming-match take — different angles.
 OK freeform quiz: 'How many players take the field for one side in cricket?'.</t>
@@ -6495,7 +7227,7 @@
           <t>SCOPE (critical): category sports means Sports (Non-Cricket) ONLY.
 NEVER mention cricket, IPL, T20, ODI, BCCI, wickets, batting, bowling, or cricket players.
 BAD sports card: 'How do you feel about the current state of Indian cricket?'.
-GOOD sports mix: football derby takes, kabaddi, badminton, hockey, F1, Olympics, chess puzzles.</t>
+GOOD sports mix: football derby takes, kabaddi, badminton, hockey, F1, Olympics, chess — rotate sports across the batch.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -6895,7 +7627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7103,7 +7835,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>BAD name spam: three cards all about Sanju Samson / Kohli / Rohit. Rotate subjects or ask knowledge questions with no star name.</t>
+          <t>Do NOT use football, kabaddi, F1, NBA, or other non-cricket sports as the primary topic.</t>
         </is>
       </c>
     </row>
@@ -7120,7 +7852,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>GOOD cricket mix: 'How many balls in an over?', 'What does DRS stand for?', one debate poll, one upcoming-match take — different angles.</t>
+          <t>BAD name spam: three cards all about Sanju Samson / Kohli / Rohit. Rotate subjects or ask knowledge questions with no star name.</t>
         </is>
       </c>
     </row>
@@ -7137,31 +7869,31 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>OK freeform quiz: 'How many players take the field for one side in cricket?'.</t>
+          <t>GOOD cricket mix: 'How many balls in an over?', 'What does DRS stand for?', one debate poll, one upcoming-match take — different angles.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>movies</t>
+          <t>cricket</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>movies</t>
+          <t>OK freeform quiz: 'How many players take the field for one side in cricket?'.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>music</t>
+          <t>movies</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -7171,14 +7903,14 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>music</t>
+          <t>movies</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>pop-culture</t>
+          <t>music</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -7188,14 +7920,14 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>pop-culture</t>
+          <t>music</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>food</t>
+          <t>pop-culture</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -7205,14 +7937,14 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>food</t>
+          <t>pop-culture</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>gaming</t>
+          <t>food</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -7222,14 +7954,14 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>gaming</t>
+          <t>food</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>sports</t>
+          <t>gaming</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -7239,7 +7971,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Sports (Non-Cricket)</t>
+          <t>gaming</t>
         </is>
       </c>
     </row>
@@ -7251,12 +7983,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>include</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>football/soccer</t>
+          <t>Sports (Non-Cricket)</t>
         </is>
       </c>
     </row>
@@ -7273,7 +8005,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>hockey</t>
+          <t>football/soccer</t>
         </is>
       </c>
     </row>
@@ -7290,7 +8022,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>badminton</t>
+          <t>hockey</t>
         </is>
       </c>
     </row>
@@ -7307,7 +8039,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>tennis</t>
+          <t>badminton</t>
         </is>
       </c>
     </row>
@@ -7324,7 +8056,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>kabaddi</t>
+          <t>tennis</t>
         </is>
       </c>
     </row>
@@ -7341,7 +8073,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>athletics</t>
+          <t>kabaddi</t>
         </is>
       </c>
     </row>
@@ -7358,7 +8090,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>athletics</t>
         </is>
       </c>
     </row>
@@ -7375,7 +8107,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>NBA / Olympics topics Indians follow</t>
+          <t>F1</t>
         </is>
       </c>
     </row>
@@ -7392,7 +8124,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>chess</t>
+          <t>NBA / Olympics topics Indians follow</t>
         </is>
       </c>
     </row>
@@ -7404,12 +8136,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>exclude</t>
+          <t>include</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>cricket</t>
+          <t>chess</t>
         </is>
       </c>
     </row>
@@ -7426,7 +8158,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>cricket</t>
         </is>
       </c>
     </row>
@@ -7443,7 +8175,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>T20</t>
+          <t>IPL</t>
         </is>
       </c>
     </row>
@@ -7460,7 +8192,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>ODI</t>
+          <t>T20</t>
         </is>
       </c>
     </row>
@@ -7477,7 +8209,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>BCCI</t>
+          <t>ODI</t>
         </is>
       </c>
     </row>
@@ -7494,7 +8226,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>wickets</t>
+          <t>BCCI</t>
         </is>
       </c>
     </row>
@@ -7511,7 +8243,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>batting/bowling cricket terms</t>
+          <t>wickets</t>
         </is>
       </c>
     </row>
@@ -7528,7 +8260,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>cricket players or Indian cricket takes</t>
+          <t>batting/bowling cricket terms</t>
         </is>
       </c>
     </row>
@@ -7540,12 +8272,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>exclude</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Cricket has its own category slug 'cricket'. Never write cricket cards for sports.</t>
+          <t>cricket players or Indian cricket takes</t>
         </is>
       </c>
     </row>
@@ -7557,12 +8289,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>note</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>SCOPE (critical): category sports means Sports (Non-Cricket) ONLY.</t>
+          <t>Cricket has its own category slug 'cricket'. Never write cricket cards for sports.</t>
         </is>
       </c>
     </row>
@@ -7579,7 +8311,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>NEVER mention cricket, IPL, T20, ODI, BCCI, wickets, batting, bowling, or cricket players.</t>
+          <t>SCOPE (critical): category sports means Sports (Non-Cricket) ONLY.</t>
         </is>
       </c>
     </row>
@@ -7596,7 +8328,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>BAD sports card: 'How do you feel about the current state of Indian cricket?'.</t>
+          <t>NEVER mention cricket, IPL, T20, ODI, BCCI, wickets, batting, bowling, or cricket players.</t>
         </is>
       </c>
     </row>
@@ -7613,31 +8345,31 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>GOOD sports mix: football derby takes, kabaddi, badminton, hockey, F1, Olympics, chess puzzles.</t>
+          <t>BAD sports card: 'How do you feel about the current state of Indian cricket?'.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>sports</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>GOOD sports mix: football derby takes, kabaddi, badminton, hockey, F1, Olympics, chess — rotate sports across the batch.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>tech</t>
+          <t>news</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -7647,14 +8379,14 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>tech</t>
+          <t>news</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>personality-vibe</t>
+          <t>tech</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -7664,14 +8396,14 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>personality-vibe</t>
+          <t>tech</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>personality-vibe</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -7681,14 +8413,14 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>personality-vibe</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -7698,14 +8430,14 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>fashion</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>kpop</t>
+          <t>health</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -7715,14 +8447,14 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>kpop</t>
+          <t>health</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>puzzles</t>
+          <t>kpop</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -7732,14 +8464,14 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>puzzles</t>
+          <t>kpop</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>logical-reasoning</t>
+          <t>puzzles</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -7749,29 +8481,46 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>logical-reasoning</t>
+          <t>puzzles</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
+          <t>logical-reasoning</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>logical-reasoning</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
           <t>math-numbers</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>math-numbers</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C51"/>
+  <autoFilter ref="A1:C52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7808,13 +8557,19 @@
   "mix": {
     "quizzes": 12,
     "polls": 8,
+    "predictionsMaxShare": 0.1,
     "preferQuizTypes": [
       "trivia",
       "who",
       "which"
+    ],
+    "preferPollTypes": [
+      "debate",
+      "hot",
+      "opinion"
     ]
   },
-  "market": "India (two layers: clean English + Gen-Z Hinglish Hindi in Devanagari; metros + Tier-2)",
+  "market": "India English feed (metros + Tier-2). Hindi/Hinglish is a separate localization stage.",
   "pollQuestionTypes": [
     "challenge",
     "company",
@@ -7850,6 +8605,27 @@
     "who"
   ],
   "evergreenBank": "Friday night. Where do you watch?\nTheatre — big screen only\nCouch and a stream\nWhat keeps you in the seat?\nAn interval twist\nA slow burn that earns the end\nA sequel is announced. You…\nBook early\nWait for reviews\nProtect the original\nInterval snack. Your move?\nAlways popcorn\nSneak your own\nSkip food\nHow do you watch?\nHindi original\nDubbed, subtitles on\nWho is in the next seat?\nThe group chat, all of them\nOne friend who will not talk\nTonight is for…\nA new Hindi release\nA rewatch of a classic\nSomeone starts a spoiler. You…\nCover your ears\nTell them to finish\nYou rewatch because…\nIt feels like home\nYou forgot the plot\nThe interval song. You…\nSing along\nWait for the story\nYou pick a film for…\nThe lead pair\nThe director\nThe credits roll. You…\nSit through them\nAre already discussing the end\nThe short break in the middle of a theatrical film in India is called the…\nInterval\nEncore\nOverture\nA film you leave the house to see on a large shared screen is a…\nTheatre screening\nDub\nSequel\nTelling the ending before someone has watched is a…\nSpoiler\nChorus\nHeadline\nPlaying a film you have already finished is a…\nRewatch\nDebut\nToss",
+  "verifiedTrends": [
+    {
+      "trendId": "movies-weekend-window",
+      "topic": "Weekend theatre release",
+      "category": "movies",
+      "freshness": "recent",
+      "eventStatus": "completed",
+      "eventDate": "2026-10-24",
+      "facts": [
+        "opening weekend",
+        "interval twist",
+        "bookings opened Thursday"
+      ],
+      "allowedAngles": [
+        "relatable consequence"
+      ],
+      "allowPrediction": false,
+      "sourceConfidence": "high",
+      "context": "This weekend's theatre release"
+    }
+  ],
   "briefs": [
     {
       "id": "movies-weekend-window",
@@ -7908,96 +8684,57 @@
     "englishGood": [
       "Midnight craving hits. Street food or Maggi at home?",
       "New trailer just dropped. Watch now or wait for friends?",
-      "Rain mid-commute. Grab a cab or tough it out?"
+      "Rain mid-commute. Grab a cab or tough it out?",
+      "DRS reviews left. Burn one now or save it?",
+      "Worth the hype or overrated — this weekend's release?"
     ],
     "englishBad": [
       "Kya scene hai for the release?",
       "Kitne excited ho for the match?",
       "What's your vibe yaar?",
-      "What is your preferred late-night dining option?"
-    ],
-    "hindiGood": [
-      {
-        "promptHi": "रात को भूख लगी — स्ट्रीट फूड या घर की मैगी?",
-        "optionsHi": [
-          "स्ट्रीट फूड 🔥",
-          "घर की मैगी"
-        ]
-      },
-      {
-        "promptHi": "नया ट्रेलर आया — क्या सीन है, अभी देखोगे?",
-        "optionsHi": [
-          "अभी स्किप मत करो",
-          "दोस्तों के साथ बाद में"
-        ]
-      },
-      {
-        "promptHi": "मैच को लेकर कितने एक्साइटेड हो?",
-        "optionsHi": [
-          "फुल ऑन! 🔥",
-          "अभी नॉर्मल हूँ"
-        ]
-      }
-    ],
-    "hindiBad": [
-      {
-        "promptHi": "What's your vibe for the trailer?",
-        "optionsHi": [
-          "Excited!",
-          "Wait and see"
-        ]
-      },
-      {
-        "promptHi": "Excited! / कितने एक्साइटेड हो?",
-        "optionsHi": [
-          "Very much",
-          "बहुत ज़्यादा"
-        ]
-      },
-      {
-        "promptHi": "Kitne excited ho for the match?",
-        "optionsHi": [
-          "Full on",
-          "Thoda sa"
-        ]
-      }
+      "What is your preferred late-night dining option?",
+      "Who is your favourite actor?",
+      "Do you like cricket?",
+      "Which do you prefer?"
     ]
   },
   "rules": [
-    "Return JSON with a candidates array.",
+    "Return JSON with a candidates array. English fields only — never promptHi, labelHi, or optionsHi.",
     "Every candidate category must equal the requested category.",
     "Stay inside categoryScope — never write a card that belongs in a different onboarding category.",
-    "Today is 2026-10-31. Every card must feel current — what India is talking about in this category right now.",
-    "MIX (critical): about 12 QUIZZES and 8 polls. Quizzes should dominate.",
+    "Today is 2026-10-31. Prefer verified live/upcoming India context from verifiedTrends when present.",
+    "Never invent a trend. Never claim something is trending without verifiedTrends / briefs support.",
+    "MIX (soft target): about 12 QUIZZES and 8 polls. Quality beats quotas — do not pad with weak cards.",
     "Prefer trivia / who / which quizzes with one clear correct answer over soft opinion polls.",
+    "Predictions: at most ~10% of the batch, and only for genuinely upcoming events with briefId.",
+    "Not formal survey speak. Not essays. Spicy but friendly. Understandable in ~3 seconds.",
+    "A quiz has exactly one correct option. Polls must set isCorrect false on every option.",
+    "Incorrect quiz options must be plausible — no absurd distractors, no 'All/None of the above'.",
+    "Two options use type predict. Three or four use type pulse.",
+    "Do not use gambling words.",
+    "INTERACTION DIVERSITY (critical): vary patterns across the batch — knowledge challenge, who/which, A vs B debate, hot take, surprising fact, upcoming prediction (only if valid), comparison, nostalgia, category-specific formats. Do not repeat the same interaction pattern.",
     "BAD batch: ten similar preference polls ('How do you watch movies?', 'Favourite snack?', 'Happy ending or cliffhanger?').",
+    "BAD lazy polls: 'Who is your favourite…?', 'Do you like X?', 'Which do you prefer?' unless timely and specific.",
+    "GOOD polls create tension, identity, disagreement, or a meaningful choice (A vs B, worth the hype?, underrated/overrated).",
+    "GOOD quizzes are knowable, surprising, recognizable, and timely when trend-based.",
     "GOOD batch: mix of fact trivia, who/which quizzes, and a few sharp debate polls on DIFFERENT topics.",
+    "One verified trend should normally produce ONE strong angle — not five paraphrases.",
+    "Possible angles when using a trend: FACT, CHOICE, DEBATE, REACTION, CONTEXT, IDENTIFY, PREDICTION (upcoming only).",
     "Write brand-new prompts. Never reuse or lightly rephrase anything in avoidPrompts.",
     "UNIQUENESS (critical): each candidate must cover a DIFFERENT topic/angle — not the same question with new wording.",
-    "NAME DIVERSITY (critical): do not reuse the same player/celebrity/team focus across multiple cards in one batch.",
-    "Knowledge trivia is encouraged: rules, formats, history, records, definitions — not only 'who is hot today' opinion polls.",
+    "NAME DIVERSITY (critical): do not reuse the same player/celebrity/team/franchise focus across multiple cards in one batch.",
+    "Treat avoidNames as a strong exclusion signal for opinion/debate focus.",
+    "Knowledge trivia is encouraged: rules, formats, history, records, definitions — not only celebrity preference polls.",
     "BAD uniqueness: 'Theatre or OTT?' and 'How do you prefer to watch films?'.",
     "Vary subjects, stakes, formats, and questionType across the batch so consecutive cards feel different.",
-    "Do not lean on the same names that already appear in avoidPrompts / avoidNames.",
-    "Prioritize India trends that are LIVE or UPCOMING for THIS category only (fixtures, releases, drops, slang, debates Indians care about). Skip party politics.",
+    "Learn from engagementInsights: copy the PATTERN of hits (format, length, debate heat); never clone exact wording; follow lessons.",
+    "Prioritize verifiedTrends that are LIVE or UPCOMING for THIS category. Skip party politics.",
     "CLOSED / PAST EVENTS (critical): NEVER ask users to predict the outcome of a match, tournament, season, election, award, or final that has already concluded as of today.",
     "BAD past prediction: 'Who will win IPL 2026?' when IPL 2026 is already over by 2026-10-31.",
     "BAD past prediction: 'Prediction: who wins the final?' for a final that already happened.",
     "OK on past events: opinion/debate only ('Fair Player of the Match?', 'Was that the right call?').",
     "OK predictions: only UPCOMING fixtures (tonight / this weekend / next match) that have not started — and only with briefId when questionType is prediction.",
     "If unsure whether an event is still open, write an opinion/debate/hot poll instead of a prediction.",
-    "Learn from engagementInsights: copy the energy of hits (format, length, debate heat); do not clone miss prompts; follow lessons.",
-    "TWO LANGUAGE LAYERS (critical): English and Hindi are separate fields — never put both in one string.",
-    "ENGLISH (prompt + option.label): natural English only. Short, second-person, swipeable. Latin script only.",
-    "NO Hinglish in English fields: never use Hindi words or Latin transliteration (yaar, kya, kitna, bahut, nahi, scene hai, full on, etc.).",
-    "English must read like English a fluent speaker would write — not Hindi written in Latin letters.",
-    "HINDI (promptHi + option.labelHi): Gen-Z Hinglish bolchal in Devanagari — how friends actually text.",
-    "Put the Hinglish energy ONLY in Hindi fields: क्या सीन है, कितने एक्साइटेड हो, वाइब, स्किप, ट्रेंड, फुल ऑन.",
-    "Hindi is NOT a word-for-word translation of the English line — rewrite the same idea with spoken Hinglish voice.",
-    "Hindi fields: Devanagari script. Keep loanwords people say (फ़िल्म, ट्रेलर, मैच, क्विज़, पोल, गेम, स्कोर, वाइब, एक्साइटेड, सीन, स्किप, रील्स, ट्रेंड, लाइक, शेयर). Do not force stiff pure-Hindi.",
-    "Never put Latin-script Hinglish or English sentences into Hindi fields (no 'Kitne excited ho', no 'Excited! / एक्साइटेड').",
-    "Short Latin acronyms/names OK inside Hindi when people keep them that way (MV, OTT, DRS, IPL).",
-    "Not formal survey speak. Not essays. Spicy but friendly.",
     "Polls use questionType opinion, debate, or hot for freeform India-trend options.",
     "Trend quizzes use questionType trivia, who, or which with STABLE well-known facts only (rules, definitions, permanent records).",
     "NEVER write a freeform quiz about who currently holds an office (CM, PM, president, captain, coach, CEO) — those need a verified briefId.",
@@ -8006,11 +8743,15 @@
     "Time-sensitive politics/news facts belong in briefs — or write an opinion/debate poll instead of a quiz.",
     "A prediction prompt must contain the word Prediction, set briefId, and the brief must allow it.",
     "Bank quizzes (evergreen types not in trendQuizTypes) must copy prompt and options from the evergreen bank.",
-    "Event copy may use only names and numbers that appear in that brief.",
-    "A quiz has exactly one correct option. Polls must set isCorrect false on every option.",
-    "Two options use type predict. Three or four use type pulse.",
-    "Do not use gambling words.",
-    "Every candidate MUST include promptHi and labelHi on every option. Never leave Hindi empty.",
+    "Event copy may use only names and numbers that appear in that brief / verified trend facts.",
+    "ENGLISH ONLY (critical): prompt and option.label must be natural English. Latin script only.",
+    "Never generate Hindi, Hinglish, Devanagari, Hindi transliteration, promptHi, labelHi, or optionsHi.",
+    "NO Hinglish in English fields: never use Hindi words or Latin transliteration (yaar, kya, kitna, bahut, nahi, scene hai, full on, etc.).",
+    "English must read like English a fluent speaker would write — not Hindi written in Latin letters.",
+    "Indian names, brand names, movie titles, and proper nouns in English are fine.",
+    "A separate Hindi localization agent will create promptHi / labelHi after validation.",
+    "Output schema per candidate: format, category, questionType, type, prompt, options[{label,isCorrect}], briefId.",
+    "Do NOT include promptHi, labelHi, or optionsHi — they are forbidden in this stage.",
     "Return about 20 candidates — fill the feed; quantity with quality."
   ]
 }</t>

</xml_diff>